<commit_message>
updated status of D_EB_11 to postiivive
</commit_message>
<xml_diff>
--- a/inst/extdata/eber_status.xlsx
+++ b/inst/extdata/eber_status.xlsx
@@ -1,42 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uvmcom-my.sharepoint.com/personal/joseph_boyd_med_uvm_edu/Documents/packages/EBVhelpR/inst/extdata/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="8_{6EE9B8A9-0463-4BAD-8A36-3EE089449EFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{657F32B5-CAA1-4551-ADF6-8A464871E8CC}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{51595F36-B3EB-4153-A86A-639069B8F07C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="109">
   <si>
     <t>EBER?</t>
   </si>
@@ -538,12 +515,19 @@
   <si>
     <t>was this miscoded or what? Now D-EB-16</t>
   </si>
+  <si>
+    <t xml:space="preserve">Positive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EBER assessed positive 2026-09-15; previously recorded as Not performed</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -553,10 +537,8 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -587,11 +569,11 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -609,10 +591,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -931,14 +909,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FDC6E82-155C-48BE-A33F-19FD6CAE47E4}">
-  <dimension ref="A1:D96"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.5703125" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -952,7 +930,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -963,7 +941,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -974,7 +952,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -985,7 +963,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -996,7 +974,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6">
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
@@ -1007,7 +985,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -1018,7 +996,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8">
       <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
@@ -1029,7 +1007,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9">
       <c r="A9" s="2" t="s">
         <v>12</v>
       </c>
@@ -1040,7 +1018,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
@@ -1051,7 +1029,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11">
       <c r="A11" s="2" t="s">
         <v>14</v>
       </c>
@@ -1062,18 +1040,21 @@
         <v>99</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12">
       <c r="A12" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>2</v>
+        <v>107</v>
       </c>
       <c r="C12" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13" s="2" t="s">
         <v>16</v>
       </c>
@@ -1084,7 +1065,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14">
       <c r="A14" s="2" t="s">
         <v>17</v>
       </c>
@@ -1095,7 +1076,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -1106,7 +1087,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16">
       <c r="A16" s="2" t="s">
         <v>19</v>
       </c>
@@ -1117,7 +1098,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17">
       <c r="A17" s="2" t="s">
         <v>94</v>
       </c>
@@ -1131,7 +1112,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18">
       <c r="A18" s="3" t="s">
         <v>103</v>
       </c>
@@ -1145,7 +1126,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -1156,7 +1137,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -1167,7 +1148,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -1178,7 +1159,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -1189,7 +1170,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -1200,7 +1181,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24">
       <c r="A24" s="2" t="s">
         <v>25</v>
       </c>
@@ -1211,7 +1192,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25">
       <c r="A25" s="2" t="s">
         <v>26</v>
       </c>
@@ -1222,7 +1203,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26">
       <c r="A26" s="2" t="s">
         <v>27</v>
       </c>
@@ -1233,7 +1214,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27">
       <c r="A27" s="2" t="s">
         <v>28</v>
       </c>
@@ -1244,7 +1225,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28">
       <c r="A28" s="2" t="s">
         <v>29</v>
       </c>
@@ -1255,7 +1236,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29">
       <c r="A29" s="2" t="s">
         <v>30</v>
       </c>
@@ -1266,7 +1247,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30">
       <c r="A30" s="2" t="s">
         <v>31</v>
       </c>
@@ -1277,7 +1258,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31">
       <c r="A31" s="2" t="s">
         <v>32</v>
       </c>
@@ -1288,7 +1269,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32">
       <c r="A32" s="2" t="s">
         <v>33</v>
       </c>
@@ -1299,7 +1280,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33">
       <c r="A33" s="2" t="s">
         <v>34</v>
       </c>
@@ -1310,7 +1291,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34">
       <c r="A34" t="s">
         <v>35</v>
       </c>
@@ -1321,7 +1302,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35">
       <c r="A35" s="2" t="s">
         <v>36</v>
       </c>
@@ -1332,7 +1313,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36">
       <c r="A36" s="2" t="s">
         <v>37</v>
       </c>
@@ -1343,7 +1324,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37">
       <c r="A37" s="2" t="s">
         <v>38</v>
       </c>
@@ -1354,7 +1335,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38">
       <c r="A38" s="2" t="s">
         <v>39</v>
       </c>
@@ -1365,7 +1346,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39">
       <c r="A39" s="2" t="s">
         <v>40</v>
       </c>
@@ -1376,7 +1357,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40">
       <c r="A40" t="s">
         <v>41</v>
       </c>
@@ -1387,7 +1368,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41">
       <c r="A41" t="s">
         <v>42</v>
       </c>
@@ -1398,7 +1379,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42">
       <c r="A42" t="s">
         <v>43</v>
       </c>
@@ -1409,7 +1390,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43">
       <c r="A43" t="s">
         <v>44</v>
       </c>
@@ -1420,7 +1401,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44">
       <c r="A44" t="s">
         <v>45</v>
       </c>
@@ -1431,7 +1412,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45">
       <c r="A45" t="s">
         <v>46</v>
       </c>
@@ -1442,7 +1423,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46">
       <c r="A46" t="s">
         <v>47</v>
       </c>
@@ -1453,7 +1434,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47">
       <c r="A47" t="s">
         <v>48</v>
       </c>
@@ -1464,7 +1445,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48">
       <c r="A48" t="s">
         <v>49</v>
       </c>
@@ -1475,7 +1456,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49">
       <c r="A49" t="s">
         <v>50</v>
       </c>
@@ -1486,7 +1467,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50">
       <c r="A50" t="s">
         <v>51</v>
       </c>
@@ -1497,7 +1478,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51">
       <c r="A51" t="s">
         <v>52</v>
       </c>
@@ -1508,7 +1489,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52">
       <c r="A52" t="s">
         <v>53</v>
       </c>
@@ -1519,7 +1500,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53">
       <c r="A53" t="s">
         <v>54</v>
       </c>
@@ -1530,7 +1511,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54">
       <c r="A54" t="s">
         <v>55</v>
       </c>
@@ -1541,7 +1522,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55">
       <c r="A55" t="s">
         <v>56</v>
       </c>
@@ -1552,7 +1533,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56">
       <c r="A56" t="s">
         <v>57</v>
       </c>
@@ -1563,7 +1544,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57">
       <c r="A57" t="s">
         <v>58</v>
       </c>
@@ -1574,7 +1555,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58">
       <c r="A58" t="s">
         <v>59</v>
       </c>
@@ -1585,7 +1566,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59">
       <c r="A59" t="s">
         <v>60</v>
       </c>
@@ -1596,7 +1577,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60">
       <c r="A60" t="s">
         <v>61</v>
       </c>
@@ -1607,7 +1588,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61">
       <c r="A61" t="s">
         <v>62</v>
       </c>
@@ -1618,7 +1599,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="62">
       <c r="A62" t="s">
         <v>63</v>
       </c>
@@ -1629,7 +1610,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="63">
       <c r="A63" t="s">
         <v>64</v>
       </c>
@@ -1640,7 +1621,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="64">
       <c r="A64" t="s">
         <v>65</v>
       </c>
@@ -1651,7 +1632,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65">
       <c r="A65" t="s">
         <v>66</v>
       </c>
@@ -1662,7 +1643,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66">
       <c r="A66" t="s">
         <v>67</v>
       </c>
@@ -1673,7 +1654,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67">
       <c r="A67" t="s">
         <v>68</v>
       </c>
@@ -1684,7 +1665,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="68">
       <c r="A68" t="s">
         <v>69</v>
       </c>
@@ -1695,7 +1676,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="69">
       <c r="A69" t="s">
         <v>70</v>
       </c>
@@ -1706,7 +1687,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="70">
       <c r="A70" t="s">
         <v>71</v>
       </c>
@@ -1717,7 +1698,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="71">
       <c r="A71" t="s">
         <v>72</v>
       </c>
@@ -1728,7 +1709,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="72">
       <c r="A72" t="s">
         <v>73</v>
       </c>
@@ -1739,7 +1720,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="73">
       <c r="A73" t="s">
         <v>74</v>
       </c>
@@ -1750,7 +1731,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="74">
       <c r="A74" t="s">
         <v>75</v>
       </c>
@@ -1761,7 +1742,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="75">
       <c r="A75" t="s">
         <v>76</v>
       </c>
@@ -1772,7 +1753,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="76">
       <c r="A76" t="s">
         <v>77</v>
       </c>
@@ -1783,7 +1764,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="77">
       <c r="A77" t="s">
         <v>78</v>
       </c>
@@ -1794,7 +1775,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="78">
       <c r="A78" t="s">
         <v>79</v>
       </c>
@@ -1805,7 +1786,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="79">
       <c r="A79" t="s">
         <v>80</v>
       </c>
@@ -1816,7 +1797,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="80">
       <c r="A80" t="s">
         <v>81</v>
       </c>
@@ -1827,7 +1808,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="81">
       <c r="A81" t="s">
         <v>82</v>
       </c>
@@ -1838,7 +1819,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82">
       <c r="A82" t="s">
         <v>83</v>
       </c>
@@ -1849,7 +1830,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83">
       <c r="A83" t="s">
         <v>84</v>
       </c>
@@ -1860,7 +1841,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84">
       <c r="A84" t="s">
         <v>85</v>
       </c>
@@ -1871,7 +1852,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85">
       <c r="A85" t="s">
         <v>86</v>
       </c>
@@ -1882,7 +1863,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86">
       <c r="A86" t="s">
         <v>87</v>
       </c>
@@ -1893,7 +1874,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87">
       <c r="A87" t="s">
         <v>88</v>
       </c>
@@ -1904,7 +1885,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88">
       <c r="A88" t="s">
         <v>89</v>
       </c>
@@ -1915,7 +1896,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89">
       <c r="A89" t="s">
         <v>90</v>
       </c>
@@ -1926,7 +1907,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90">
       <c r="A90" t="s">
         <v>91</v>
       </c>
@@ -1937,7 +1918,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91">
       <c r="A91" t="s">
         <v>92</v>
       </c>
@@ -1948,7 +1929,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92">
       <c r="A92" t="s">
         <v>93</v>
       </c>
@@ -1959,7 +1940,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93">
       <c r="A93" t="s">
         <v>95</v>
       </c>
@@ -1970,7 +1951,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94">
       <c r="A94" t="s">
         <v>96</v>
       </c>
@@ -1981,7 +1962,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95">
       <c r="A95" t="s">
         <v>97</v>
       </c>
@@ -1992,7 +1973,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96">
       <c r="A96" t="s">
         <v>101</v>
       </c>
@@ -2005,5 +1986,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>